<commit_message>
feat: implement Inventory & ExpiryReports modules and major refactoring
- Added full Inventory features (`AdjustStock`, `UpdateStock`, `ToggleRare`).
- Created complete `ExpiryReport` module (Log, Revert, GetAll) with automatic stock adjustments.
- Refactored multiple Handlers to use `GetAsync` for PKs and modern pattern matching (`is not { }`).
- Renamed `IsManualShortage` to `IsRare` and synced EF Core migrations.
- Fixed `FakeItEasy` nullable warnings in tests and resolved OpenAPI Source Generator build error.
- Massively updated `AGENTS.md` and `tasks.md` with new architectural rules and tracking.
</commit_message>
<xml_diff>
--- a/PharmaSaaS_SystemAnalysis.xlsx
+++ b/PharmaSaaS_SystemAnalysis.xlsx
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>GET /api/lookups/categories</t>
+          <t>GET /api/Categories</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>POST /api/lookups/categories</t>
+          <t>POST /api/Categories</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>GET /api/lookups/dosage-forms</t>
+          <t>GET /api/DosageForms</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>POST /api/lookups/dosage-forms</t>
+          <t>POST /api/DosageForms</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>GET /api/employees</t>
+          <t>GET /api/Users</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>POST /api/employees</t>
+          <t>POST /api/Users</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>PUT /api/employees/{id}</t>
+          <t>PUT /api/Users/{id}</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>DELETE /api/employees/{id}</t>
+          <t>DELETE /api/Users/{id}</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -4076,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4160,19 +4160,18 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>[{ product, quantity, purchasePrice, targetStock, isManualShortage, isAutoShortage }]</t>
+          <t>[{ product, quantity, purchasePrice, targetStock, isRare }]</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Returns current stock levels per product per branch.</t>
+          <t>Returns current stock levels per product. isRare flags products rare in the market.</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
           <t>1. Extract PharmacyId from JWT
-2. Calculate isAutoShortage (quantity &lt;= 25% of targetStock)
-3. Return results</t>
+2. Return all inventory records</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -4220,10 +4219,7 @@
       <c r="G3" s="7" t="inlineStr">
         <is>
           <t>1. Validate product belongs to pharmacy
-2. Update inventory record
-3. Recalculate isAutoShortage flag
-4. If quantity &lt;= 50% targetStock → add to low-stock watch list
-5. If quantity &lt;= 25% targetStock → set isAutoShortage = true</t>
+2. Update inventory record</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -4240,7 +4236,7 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Toggle Manual Shortage</t>
+          <t>Toggle Rare Flag</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -4255,7 +4251,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>{ isManualShortage: bool }</t>
+          <t>- (no body, toggles the flag automatically)</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -4265,13 +4261,13 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Manually flags or unflags a product as unavailable regardless of quantity.</t>
+          <t>Toggles the isRare flag for a product. Marks product as rare/scarce in the market regardless of stock quantity.</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
           <t>1. Validate product belongs to pharmacy
-2. Update isManualShortage flag</t>
+2. Toggle isRare flag</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -4288,7 +4284,7 @@
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Shortage Report</t>
+          <t>Rare Products Report</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -4308,18 +4304,18 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>[{ product, quantity, targetStock, isManualShortage, isAutoShortage }]</t>
+          <t>[{ product, quantity, targetStock, isRare }]</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Returns all products currently flagged as shortage — either auto (&lt;=25% target) or manual.</t>
+          <t>Returns all products currently flagged as rare in the market (isRare = true).</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
           <t>1. Extract PharmacyId
-2. Filter products where isAutoShortage=true OR isManualShortage=true
+2. Filter products where isRare = true
 3. Return list</t>
         </is>
       </c>
@@ -4337,50 +4333,147 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>Stock Level Report</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Manager / Owner</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>GET /api/inventory/stock-level?belowTarget={bool}</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>belowTarget: bool (query param)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>[{ product, quantity, targetStock, isRare }]</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Returns products filtered by stock level relative to their target. Only products with a configured targetStock are included.</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>1. Extract PharmacyId
+2. Filter: targetStock set AND (quantity &lt; targetStock if belowTarget=true, else quantity &gt;= targetStock)
+3. Return list</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Owner, Manager, Pharmacist</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Management / Procurement Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Out-of-Stock Report</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Manager / Owner</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>GET /api/inventory/out-of-stock</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>— (PharmacyId from JWT)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>[{ product, quantity, targetStock, isRare }]</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Returns all products with zero quantity (completely out of stock).</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>1. Extract PharmacyId
+2. Filter products where quantity = 0
+3. Return list</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Owner, Manager, Pharmacist</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Management / Procurement Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
           <t>Log Expiry Report</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Pharmacist</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>POST /api/inventory/expiry-report</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>{ productId, expiredQuantity, notes? }</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>{ id }</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>204 No Content</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Records expired stock and automatically deducts the expired quantity from inventory.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>1. Validate product belongs to pharmacy
 2. Check expiredQuantity &lt;= current quantity
 3. Create ExpiryReport record
 4. Deduct expiredQuantity from Inventory.Quantity
-5. Recalculate shortage flags
-6. Return report id</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
+5. Return 204</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Owner, Manager, Pharmacist</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Pharmacy System / Audit Log</t>
         </is>

</xml_diff>